<commit_message>
refactor(stock_item): restructure module and add delete, update, and export methods
</commit_message>
<xml_diff>
--- a/PizzaroGoApp/ExcelFileForApp/Stock.xlsx
+++ b/PizzaroGoApp/ExcelFileForApp/Stock.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\stoic\Desktop\Academy\Project\PizzaroGo\PizzaroGoApp\ExcelFileForApp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{05D024AA-A3EE-4474-B79A-B9A141557384}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3564DE46-CBC2-4C99-84DF-76C4D33E3223}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="57480" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="15">
   <si>
     <t>Name</t>
   </si>
@@ -64,6 +64,15 @@
   </si>
   <si>
     <t>l</t>
+  </si>
+  <si>
+    <t>Category</t>
+  </si>
+  <si>
+    <t>Ingerdient</t>
+  </si>
+  <si>
+    <t>Product</t>
   </si>
 </sst>
 </file>
@@ -381,86 +390,107 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C7"/>
+  <dimension ref="A1:D7"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="16.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
+        <v>12</v>
+      </c>
+      <c r="C1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>3</v>
       </c>
-      <c r="B2">
+      <c r="B2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C2">
         <v>200</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>5</v>
       </c>
-      <c r="B3">
+      <c r="B3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C3">
         <v>200</v>
       </c>
-      <c r="C3" t="s">
+      <c r="D3" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>6</v>
       </c>
-      <c r="B4">
+      <c r="B4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C4">
         <v>500</v>
       </c>
-      <c r="C4" t="s">
+      <c r="D4" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>8</v>
       </c>
-      <c r="B5">
+      <c r="B5" t="s">
+        <v>13</v>
+      </c>
+      <c r="C5">
         <v>700</v>
       </c>
-      <c r="C5" t="s">
+      <c r="D5" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>9</v>
       </c>
-      <c r="B6">
+      <c r="B6" t="s">
+        <v>13</v>
+      </c>
+      <c r="C6">
         <v>800</v>
       </c>
-      <c r="C6" t="s">
+      <c r="D6" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>10</v>
       </c>
-      <c r="B7">
+      <c r="B7" t="s">
+        <v>13</v>
+      </c>
+      <c r="C7">
         <v>700</v>
       </c>
-      <c r="C7" t="s">
+      <c r="D7" t="s">
         <v>7</v>
       </c>
     </row>

</xml_diff>

<commit_message>
refactor(stock_item):  updated frontend structure to match backend modifications introduced in the previous commit
</commit_message>
<xml_diff>
--- a/PizzaroGoApp/ExcelFileForApp/Stock.xlsx
+++ b/PizzaroGoApp/ExcelFileForApp/Stock.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\stoic\Desktop\Academy\Project\PizzaroGo\PizzaroGoApp\ExcelFileForApp\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3564DE46-CBC2-4C99-84DF-76C4D33E3223}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF13AB4F-209A-4368-B087-BD6F0253B647}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -69,10 +69,10 @@
     <t>Category</t>
   </si>
   <si>
-    <t>Ingerdient</t>
-  </si>
-  <si>
     <t>Product</t>
+  </si>
+  <si>
+    <t>Ingredient</t>
   </si>
 </sst>
 </file>
@@ -415,7 +415,7 @@
         <v>3</v>
       </c>
       <c r="B2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C2">
         <v>200</v>
@@ -429,7 +429,7 @@
         <v>5</v>
       </c>
       <c r="B3" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C3">
         <v>200</v>
@@ -443,7 +443,7 @@
         <v>6</v>
       </c>
       <c r="B4" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C4">
         <v>500</v>
@@ -457,7 +457,7 @@
         <v>8</v>
       </c>
       <c r="B5" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C5">
         <v>700</v>
@@ -471,7 +471,7 @@
         <v>9</v>
       </c>
       <c r="B6" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C6">
         <v>800</v>
@@ -485,7 +485,7 @@
         <v>10</v>
       </c>
       <c r="B7" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C7">
         <v>700</v>

</xml_diff>